<commit_message>
Add crosscheck table display to review.py output
- Added print_crosscheck_table() function to display detailed prediction vs actual results
- Shows prediction strings, actual results with hit indicators, and hit counts per race
- Displays above the accuracy report in review.py console output
- Matches the requested format with horse numbers and checkmarks for hits
</commit_message>
<xml_diff>
--- a/data/results/2026-03-25_HV.xlsx
+++ b/data/results/2026-03-25_HV.xlsx
@@ -11835,7 +11835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11879,6 +11879,21 @@
           <t>margin</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -11917,6 +11932,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -11955,6 +11973,9 @@
           <t>N</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -11993,6 +12014,9 @@
           <t>1</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -12031,6 +12055,9 @@
           <t>1-3/4</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -12069,6 +12096,9 @@
           <t>2</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -12107,6 +12137,9 @@
           <t>2-1/4</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -12145,6 +12178,9 @@
           <t>3</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -12183,6 +12219,9 @@
           <t>3</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -12221,6 +12260,9 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -12259,6 +12301,9 @@
           <t>6-3/4</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -12297,6 +12342,9 @@
           <t>8</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -12335,6 +12383,9 @@
           <t>10</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12347,7 +12398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12391,6 +12442,21 @@
           <t>margin</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -12429,6 +12495,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -12467,6 +12536,9 @@
           <t>NOSE</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -12505,6 +12577,9 @@
           <t>2-1/4</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -12543,6 +12618,9 @@
           <t>3</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -12581,6 +12659,9 @@
           <t>3-1/2</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -12619,6 +12700,9 @@
           <t>4-1/4</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -12657,6 +12741,9 @@
           <t>4-1/4</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -12695,6 +12782,9 @@
           <t>5-3/4</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -12733,6 +12823,9 @@
           <t>5-3/4</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -12771,6 +12864,9 @@
           <t>8-1/4</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -12809,6 +12905,9 @@
           <t>9-1/4</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -12847,6 +12946,9 @@
           <t>11-1/4</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12859,7 +12961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12903,6 +13005,21 @@
           <t>margin</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -12941,6 +13058,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -12979,6 +13099,9 @@
           <t>1/2</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -13017,6 +13140,9 @@
           <t>3/4</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -13055,6 +13181,9 @@
           <t>1-1/4</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -13093,6 +13222,9 @@
           <t>1-3/4</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -13131,6 +13263,9 @@
           <t>2-1/2</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -13169,6 +13304,9 @@
           <t>2-3/4</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -13207,6 +13345,9 @@
           <t>2-3/4</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -13245,6 +13386,9 @@
           <t>3-1/4</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -13283,6 +13427,9 @@
           <t>5-1/2</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -13321,6 +13468,9 @@
           <t>6-3/4</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -13359,6 +13509,9 @@
           <t>8-3/4</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13371,7 +13524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13415,6 +13568,21 @@
           <t>margin</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -13453,6 +13621,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -13491,6 +13662,9 @@
           <t>HD</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -13529,6 +13703,9 @@
           <t>3/4</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -13567,6 +13744,9 @@
           <t>1-1/4</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -13605,6 +13785,9 @@
           <t>1-1/4</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -13643,6 +13826,9 @@
           <t>2-1/2</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -13681,6 +13867,9 @@
           <t>3-1/4</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -13719,6 +13908,9 @@
           <t>3-3/4</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -13757,6 +13949,9 @@
           <t>4</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -13795,6 +13990,9 @@
           <t>5</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -13833,6 +14031,9 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -13871,6 +14072,9 @@
           <t>8-3/4</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13883,7 +14087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13927,6 +14131,21 @@
           <t>margin</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -13965,6 +14184,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -14003,6 +14225,9 @@
           <t>3/4</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -14041,6 +14266,9 @@
           <t>1-3/4</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -14079,6 +14307,9 @@
           <t>2</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -14117,6 +14348,9 @@
           <t>2</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -14155,6 +14389,9 @@
           <t>2-3/4</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -14193,6 +14430,9 @@
           <t>3</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -14231,6 +14471,9 @@
           <t>4</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -14269,6 +14512,9 @@
           <t>5-1/4</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -14307,6 +14553,9 @@
           <t>7-1/2</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -14345,6 +14594,9 @@
           <t>10-1/4</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -14383,6 +14635,9 @@
           <t>24-3/4</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14395,7 +14650,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14439,6 +14694,21 @@
           <t>margin</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -14477,6 +14747,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -14515,6 +14788,9 @@
           <t>3/4</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -14553,6 +14829,9 @@
           <t>3/4</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -14591,6 +14870,9 @@
           <t>3/4</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -14629,6 +14911,9 @@
           <t>3/4</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -14667,6 +14952,9 @@
           <t>2-1/4</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -14705,6 +14993,9 @@
           <t>3-3/4</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -14743,6 +15034,9 @@
           <t>4</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -14781,6 +15075,9 @@
           <t>4-1/4</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -14819,6 +15116,9 @@
           <t>4-1/2</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -14857,6 +15157,9 @@
           <t>12</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -14895,6 +15198,9 @@
           <t>---</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14907,7 +15213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -14951,6 +15257,21 @@
           <t>margin</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -14989,6 +15310,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -15027,6 +15351,9 @@
           <t>SH</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -15065,6 +15392,9 @@
           <t>1-1/2</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -15103,6 +15433,9 @@
           <t>2-1/4</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -15141,6 +15474,9 @@
           <t>2-3/4</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -15179,6 +15515,9 @@
           <t>4-1/2</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -15217,6 +15556,9 @@
           <t>4-1/2</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -15255,6 +15597,9 @@
           <t>4-3/4</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -15293,6 +15638,9 @@
           <t>5-3/4</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -15331,6 +15679,9 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -15369,6 +15720,9 @@
           <t>6-1/4</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -15407,6 +15761,9 @@
           <t>---</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15419,7 +15776,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15463,6 +15820,21 @@
           <t>margin</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -15501,6 +15873,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -15539,6 +15914,9 @@
           <t>3</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -15577,6 +15955,9 @@
           <t>4-1/2</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -15615,6 +15996,9 @@
           <t>5</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -15653,6 +16037,9 @@
           <t>5-1/4</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -15691,6 +16078,9 @@
           <t>5-1/2</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -15729,6 +16119,9 @@
           <t>5-3/4</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -15767,6 +16160,9 @@
           <t>6-1/2</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -15805,6 +16201,9 @@
           <t>6-1/2</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -15843,6 +16242,9 @@
           <t>7-1/2</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -15881,6 +16283,9 @@
           <t>8-1/2</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -15919,6 +16324,9 @@
           <t>10-1/2</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15931,7 +16339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15975,6 +16383,21 @@
           <t>margin</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -16013,6 +16436,9 @@
           <t>-</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -16051,6 +16477,9 @@
           <t>N</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -16089,6 +16518,9 @@
           <t>1/2</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -16127,6 +16559,9 @@
           <t>2-3/4</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -16165,6 +16600,9 @@
           <t>4-1/4</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -16203,6 +16641,9 @@
           <t>4-3/4</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -16241,6 +16682,9 @@
           <t>5</t>
         </is>
       </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -16279,6 +16723,9 @@
           <t>5-1/2</t>
         </is>
       </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -16317,6 +16764,9 @@
           <t>7-3/4</t>
         </is>
       </c>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -16355,6 +16805,9 @@
           <t>10</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -16393,6 +16846,9 @@
           <t>10-1/2</t>
         </is>
       </c>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -16431,6 +16887,9 @@
           <t>14-1/2</t>
         </is>
       </c>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -16465,6 +16924,9 @@
           <t>---</t>
         </is>
       </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>